<commit_message>
Run every tool call of a reply in order; clarify template rules; lab reruns by values
The Gateway refused a reply carrying several tool calls and ended the
turn (lab fix-002 X02); each call now runs in order against the turn's
budget and gets its tool message. Templates' Instructions now say layout
(column widths, freeze, filters, styles) stays as is and a value the
source lacks stays blank. The lab's rerun request names new values only
and grades the workbook the rerun wrote, keeping the first result aside.
The coding runner gains tzdata (Asia/Taipei for zoneinfo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/business_workflow_lab/templates/expense_template.xlsx
+++ b/benchmarks/business_workflow_lab/templates/expense_template.xlsx
@@ -834,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1044,46 +1044,46 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AmountTWD</t>
+          <t>Layout</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>原幣金額 × 匯率（fx_rates.csv），四捨五入 ROUND_HALF_UP 至兩位小數；不同幣別的原幣金額不可直接相加。</t>
+          <t>欄寬、凍結窗格、自動篩選、字型與填色保留模板設定，不要調整或自動調整欄寬。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>All detail sheets</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>Missing values</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>ExpenseID: text (文字，保留前導零)</t>
+          <t>來源沒有的值留空（空白儲存格），不要填 N/A、0 或自行推測的值。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Details</t>
+          <t>All sheets</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>AmountTWD</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>EmployeeID: text (文字，保留前導零)</t>
+          <t>原幣金額 × 匯率（fx_rates.csv），四捨五入 ROUND_HALF_UP 至兩位小數；不同幣別的原幣金額不可直接相加。</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1095,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>EmployeeName: text</t>
+          <t>ExpenseID: text (文字，保留前導零)</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1112,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>ProjectID: text (文字，保留前導零)</t>
+          <t>EmployeeID: text (文字，保留前導零)</t>
         </is>
       </c>
     </row>
@@ -1129,12 +1129,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>ExpenseDate: date YYYY-MM-DD</t>
+          <t>EmployeeName: text</t>
         </is>
       </c>
     </row>
@@ -1146,12 +1146,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Category: text</t>
+          <t>ProjectID: text (文字，保留前導零)</t>
         </is>
       </c>
     </row>
@@ -1163,12 +1163,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Currency: text</t>
+          <t>ExpenseDate: date YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>H4</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Amount: number, 2 decimals (0.00)</t>
+          <t>Category: text</t>
         </is>
       </c>
     </row>
@@ -1197,12 +1197,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>AmountTWD: number, 2 decimals (0.00)</t>
+          <t>Currency: text</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>H4</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Status: text</t>
+          <t>Amount: number, 2 decimals (0.00)</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1231,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>ReceiptID: text (文字，保留前導零)</t>
+          <t>AmountTWD: number, 2 decimals (0.00)</t>
         </is>
       </c>
     </row>
@@ -1248,12 +1248,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>L4</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Description: text</t>
+          <t>Status: text</t>
         </is>
       </c>
     </row>
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>MissingReceipt: text</t>
+          <t>ReceiptID: text (文字，保留前導零)</t>
         </is>
       </c>
     </row>
@@ -1282,12 +1282,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>N4</t>
+          <t>L4</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>NeedsReview: text</t>
+          <t>Description: text</t>
         </is>
       </c>
     </row>
@@ -1299,61 +1299,95 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>M / N</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>MissingReceipt、NeedsReview 填 true 或 false（布林值或文字 true/false）。</t>
+          <t>MissingReceipt: text</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Details</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>N4</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>公式 =SUM(Details!I5:I{最後資料列})：Details 的 AmountTWD 合計；填入資料後把範圍延伸到最後一列，零筆時保留 I5:I5。</t>
+          <t>NeedsReview: text</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Details</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>A4:F4 / row 5+</t>
+          <t>M / N</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>彙總表：Group、SubGroup 為分組鍵（依題目要求，例如 Status、Currency、EmployeeID、Category；不用時留空），Currency 為原幣，Amount 為該組原幣合計，AmountTWD 為該組 TWD 合計，Count 為筆數；全部 TWD 總額不得混加不同原幣。</t>
+          <t>MissingReceipt、NeedsReview 填 true 或 false（布林值或文字 true/false）。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>公式 =SUM(Details!I5:I{最後資料列})：Details 的 AmountTWD 合計；填入資料後把範圍延伸到最後一列，零筆時保留 I5:I5。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>A4:F4 / row 5+</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>彙總表：Group、SubGroup 為分組鍵（依題目要求，例如 Status、Currency、EmployeeID、Category；不用時留空），Currency 為原幣，Amount 為該組原幣合計，AmountTWD 為該組 TWD 合計，Count 為筆數；全部 TWD 總額不得混加不同原幣。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Exceptions</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>A4:D4 / row 5+</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>例外清單：原始 ExpenseID、EmployeeID、ExpenseDate 與原因；列入例外的費用仍須保留在 Details。</t>
         </is>

</xml_diff>